<commit_message>
Final Changes (I hope)
</commit_message>
<xml_diff>
--- a/data/Macro_Data.xlsx
+++ b/data/Macro_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diaz/Documents/Masters/Coursework/First Semester/Macroeconomics/Project/Macro Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D692FC-27E5-7A43-BBE4-AE1C876381BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C236FA7D-C17E-5B43-B5C3-5C8C022441F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15920" activeTab="5" xr2:uid="{FACA270E-A051-484D-8F71-78DED5343A90}"/>
   </bookViews>
@@ -8107,7 +8107,7 @@
       </c>
       <c r="E2" s="23">
         <f>Inflation!C6</f>
-        <v>7.5819089534076928E-2</v>
+        <v>8.8837224183347923E-3</v>
       </c>
       <c r="F2" s="23">
         <f>Federal_Funds_Effective_Rate!C2</f>
@@ -8132,7 +8132,7 @@
       </c>
       <c r="E3" s="23">
         <f>Inflation!C7</f>
-        <v>6.9067697483485055E-2</v>
+        <v>1.4450317124735778E-2</v>
       </c>
       <c r="F3" s="23">
         <f>Federal_Funds_Effective_Rate!C3</f>
@@ -8157,7 +8157,7 @@
       </c>
       <c r="E4" s="23">
         <f>Inflation!C8</f>
-        <v>5.8157304344998752E-2</v>
+        <v>1.7360134212802285E-2</v>
       </c>
       <c r="F4" s="23">
         <f>Federal_Funds_Effective_Rate!C4</f>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="E5" s="23">
         <f>Inflation!C9</f>
-        <v>4.4429276824469281E-2</v>
+        <v>3.0727315559289522E-3</v>
       </c>
       <c r="F5" s="23">
         <f>Federal_Funds_Effective_Rate!C5</f>
@@ -8207,7 +8207,7 @@
       </c>
       <c r="E6" s="23">
         <f>Inflation!C10</f>
-        <v>3.5940803382663908E-2</v>
+        <v>6.841411985744648E-4</v>
       </c>
       <c r="F6" s="23">
         <f>Federal_Funds_Effective_Rate!C6</f>
@@ -8232,7 +8232,7 @@
       </c>
       <c r="E7" s="23">
         <f>Inflation!C11</f>
-        <v>3.2990507153500652E-2</v>
+        <v>1.1561224489795872E-2</v>
       </c>
       <c r="F7" s="23">
         <f>Federal_Funds_Effective_Rate!C7</f>
@@ -8257,7 +8257,7 @@
       </c>
       <c r="E8" s="23">
         <f>Inflation!C12</f>
-        <v>2.5268095828254778E-2</v>
+        <v>9.7545721404577561E-3</v>
       </c>
       <c r="F8" s="23">
         <f>Federal_Funds_Effective_Rate!C8</f>
@@ -8282,7 +8282,7 @@
       </c>
       <c r="E9" s="23">
         <f>Inflation!C13</f>
-        <v>3.2338435460978296E-2</v>
+        <v>9.99000999000999E-3</v>
       </c>
       <c r="F9" s="23">
         <f>Federal_Funds_Effective_Rate!C9</f>
@@ -8307,7 +8307,7 @@
       </c>
       <c r="E10" s="23">
         <f>Inflation!C14</f>
-        <v>4.6255102040816343E-2</v>
+        <v>1.4174085064292848E-2</v>
       </c>
       <c r="F10" s="23">
         <f>Federal_Funds_Effective_Rate!C10</f>
@@ -8332,7 +8332,7 @@
       </c>
       <c r="E11" s="23">
         <f>Inflation!C15</f>
-        <v>4.4051930235138696E-2</v>
+        <v>9.4311099841026674E-3</v>
       </c>
       <c r="F11" s="23">
         <f>Federal_Funds_Effective_Rate!C11</f>
@@ -8357,7 +8357,7 @@
       </c>
       <c r="E12" s="23">
         <f>Inflation!C16</f>
-        <v>4.2957042957043071E-2</v>
+        <v>8.6956521739130991E-3</v>
       </c>
       <c r="F12" s="23">
         <f>Federal_Funds_Effective_Rate!C12</f>
@@ -8382,7 +8382,7 @@
       </c>
       <c r="E13" s="23">
         <f>Inflation!C17</f>
-        <v>4.1543026706231487E-2</v>
+        <v>8.6206896551723321E-3</v>
       </c>
       <c r="F13" s="23">
         <f>Federal_Funds_Effective_Rate!C13</f>
@@ -8407,7 +8407,7 @@
       </c>
       <c r="E14" s="23">
         <f>Inflation!C18</f>
-        <v>3.6417543620102744E-2</v>
+        <v>9.1832858499525053E-3</v>
       </c>
       <c r="F14" s="23">
         <f>Federal_Funds_Effective_Rate!C14</f>
@@ -8432,7 +8432,7 @@
       </c>
       <c r="E15" s="23">
         <f>Inflation!C19</f>
-        <v>3.6067632850241588E-2</v>
+        <v>9.0903102562414316E-3</v>
       </c>
       <c r="F15" s="23">
         <f>Federal_Funds_Effective_Rate!C15</f>
@@ -8457,7 +8457,7 @@
       </c>
       <c r="E16" s="23">
         <f>Inflation!C20</f>
-        <v>3.3524904214559385E-2</v>
+        <v>6.2201001557356554E-3</v>
       </c>
       <c r="F16" s="23">
         <f>Federal_Funds_Effective_Rate!C16</f>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="E17" s="23">
         <f>Inflation!C21</f>
-        <v>3.5137701804368496E-2</v>
+        <v>1.0194624652455924E-2</v>
       </c>
       <c r="F17" s="23">
         <f>Federal_Funds_Effective_Rate!C17</f>
@@ -8507,7 +8507,7 @@
       </c>
       <c r="E18" s="23">
         <f>Inflation!C22</f>
-        <v>3.105385491262572E-2</v>
+        <v>5.2018348623852576E-3</v>
       </c>
       <c r="F18" s="23">
         <f>Federal_Funds_Effective_Rate!C18</f>
@@ -8532,7 +8532,7 @@
       </c>
       <c r="E19" s="23">
         <f>Inflation!C23</f>
-        <v>1.6785877481745332E-2</v>
+        <v>-4.873730228992232E-3</v>
       </c>
       <c r="F19" s="23">
         <f>Federal_Funds_Effective_Rate!C19</f>
@@ -8557,7 +8557,7 @@
       </c>
       <c r="E20" s="23">
         <f>Inflation!C24</f>
-        <v>1.668211306765521E-2</v>
+        <v>6.1174139939284581E-3</v>
       </c>
       <c r="F20" s="23">
         <f>Federal_Funds_Effective_Rate!C20</f>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="E21" s="23">
         <f>Inflation!C25</f>
-        <v>1.3458715596330264E-2</v>
+        <v>6.9917958067456324E-3</v>
       </c>
       <c r="F21" s="23">
         <f>Federal_Funds_Effective_Rate!C21</f>
@@ -8607,7 +8607,7 @@
       </c>
       <c r="E22" s="23">
         <f>Inflation!C26</f>
-        <v>2.0380223972546518E-2</v>
+        <v>1.2066952121448021E-2</v>
       </c>
       <c r="F22" s="23">
         <f>Federal_Funds_Effective_Rate!C22</f>
@@ -8632,7 +8632,7 @@
       </c>
       <c r="E23" s="23">
         <f>Inflation!C27</f>
-        <v>3.6997973090715577E-2</v>
+        <v>1.1332737030411412E-2</v>
       </c>
       <c r="F23" s="23">
         <f>Federal_Funds_Effective_Rate!C23</f>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="E24" s="23">
         <f>Inflation!C28</f>
-        <v>4.1631722880583345E-2</v>
+        <v>1.0613176258324735E-2</v>
       </c>
       <c r="F24" s="23">
         <f>Federal_Funds_Effective_Rate!C24</f>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="E25" s="23">
         <f>Inflation!C29</f>
-        <v>4.4049354105751039E-2</v>
+        <v>9.3290276282741516E-3</v>
       </c>
       <c r="F25" s="23">
         <f>Federal_Funds_Effective_Rate!C25</f>
@@ -8707,7 +8707,7 @@
       </c>
       <c r="E26" s="23">
         <f>Inflation!C30</f>
-        <v>3.965116279069774E-2</v>
+        <v>7.8034907615340422E-3</v>
       </c>
       <c r="F26" s="23">
         <f>Federal_Funds_Effective_Rate!C26</f>
@@ -8732,7 +8732,7 @@
       </c>
       <c r="E27" s="23">
         <f>Inflation!C31</f>
-        <v>3.9799410968717662E-2</v>
+        <v>1.147694716646726E-2</v>
       </c>
       <c r="F27" s="23">
         <f>Federal_Funds_Effective_Rate!C27</f>
@@ -8757,7 +8757,7 @@
       </c>
       <c r="E28" s="23">
         <f>Inflation!C32</f>
-        <v>4.1420532612215288E-2</v>
+        <v>1.2188794474640052E-2</v>
       </c>
       <c r="F28" s="23">
         <f>Federal_Funds_Effective_Rate!C28</f>
@@ -8782,7 +8782,7 @@
       </c>
       <c r="E29" s="23">
         <f>Inflation!C33</f>
-        <v>4.3066598458377035E-2</v>
+        <v>1.0924369747899136E-2</v>
       </c>
       <c r="F29" s="23">
         <f>Federal_Funds_Effective_Rate!C29</f>
@@ -8807,7 +8807,7 @@
       </c>
       <c r="E30" s="23">
         <f>Inflation!C34</f>
-        <v>4.6750922715579887E-2</v>
+        <v>1.136325852036579E-2</v>
       </c>
       <c r="F30" s="23">
         <f>Federal_Funds_Effective_Rate!C30</f>
@@ -8832,7 +8832,7 @@
       </c>
       <c r="E31" s="23">
         <f>Inflation!C35</f>
-        <v>5.1596111153640073E-2</v>
+        <v>1.6158859838740117E-2</v>
       </c>
       <c r="F31" s="23">
         <f>Federal_Funds_Effective_Rate!C31</f>
@@ -8857,7 +8857,7 @@
       </c>
       <c r="E32" s="23">
         <f>Inflation!C36</f>
-        <v>4.7058823529411715E-2</v>
+        <v>7.8215363212087285E-3</v>
       </c>
       <c r="F32" s="23">
         <f>Federal_Funds_Effective_Rate!C32</f>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="E33" s="23">
         <f>Inflation!C37</f>
-        <v>4.6275976724854589E-2</v>
+        <v>1.0168539325842779E-2</v>
       </c>
       <c r="F33" s="23">
         <f>Federal_Funds_Effective_Rate!C33</f>
@@ -8907,7 +8907,7 @@
       </c>
       <c r="E34" s="23">
         <f>Inflation!C38</f>
-        <v>5.2323144320152427E-2</v>
+        <v>1.7208640866946717E-2</v>
       </c>
       <c r="F34" s="23">
         <f>Federal_Funds_Effective_Rate!C34</f>
@@ -8932,7 +8932,7 @@
       </c>
       <c r="E35" s="23">
         <f>Inflation!C39</f>
-        <v>4.5837276455315455E-2</v>
+        <v>9.8958862168349142E-3</v>
       </c>
       <c r="F35" s="23">
         <f>Federal_Funds_Effective_Rate!C35</f>
@@ -8957,7 +8957,7 @@
       </c>
       <c r="E36" s="23">
         <f>Inflation!C40</f>
-        <v>5.5642054574638791E-2</v>
+        <v>1.7269914926527265E-2</v>
       </c>
       <c r="F36" s="23">
         <f>Federal_Funds_Effective_Rate!C36</f>
@@ -8982,7 +8982,7 @@
       </c>
       <c r="E37" s="23">
         <f>Inflation!C41</f>
-        <v>6.2764664288494934E-2</v>
+        <v>1.6984330928360252E-2</v>
       </c>
       <c r="F37" s="23">
         <f>Federal_Funds_Effective_Rate!C37</f>
@@ -9007,7 +9007,7 @@
       </c>
       <c r="E38" s="23">
         <f>Inflation!C42</f>
-        <v>5.259581514140893E-2</v>
+        <v>7.4756853334529442E-3</v>
       </c>
       <c r="F38" s="23">
         <f>Federal_Funds_Effective_Rate!C38</f>
@@ -9032,7 +9032,7 @@
       </c>
       <c r="E39" s="23">
         <f>Inflation!C43</f>
-        <v>4.8468677494199502E-2</v>
+        <v>5.9361713179043188E-3</v>
       </c>
       <c r="F39" s="23">
         <f>Federal_Funds_Effective_Rate!C39</f>
@@ -9057,7 +9057,7 @@
       </c>
       <c r="E40" s="23">
         <f>Inflation!C44</f>
-        <v>3.8522652110116913E-2</v>
+        <v>7.6198484882013104E-3</v>
       </c>
       <c r="F40" s="23">
         <f>Federal_Funds_Effective_Rate!C40</f>
@@ -9082,7 +9082,7 @@
       </c>
       <c r="E41" s="23">
         <f>Inflation!C45</f>
-        <v>2.964856803247444E-2</v>
+        <v>8.2942898975110532E-3</v>
       </c>
       <c r="F41" s="23">
         <f>Federal_Funds_Effective_Rate!C41</f>
@@ -9107,7 +9107,7 @@
       </c>
       <c r="E42" s="23">
         <f>Inflation!C46</f>
-        <v>2.8938835174783187E-2</v>
+        <v>6.7812361598164382E-3</v>
       </c>
       <c r="F42" s="23">
         <f>Federal_Funds_Effective_Rate!C42</f>
@@ -9132,7 +9132,7 @@
       </c>
       <c r="E43" s="23">
         <f>Inflation!C47</f>
-        <v>3.0730192450965182E-2</v>
+        <v>7.6874815204771322E-3</v>
       </c>
       <c r="F43" s="23">
         <f>Federal_Funds_Effective_Rate!C43</f>
@@ -9157,7 +9157,7 @@
       </c>
       <c r="E44" s="23">
         <f>Inflation!C48</f>
-        <v>3.0746705710102615E-2</v>
+        <v>7.6359914980713732E-3</v>
       </c>
       <c r="F44" s="23">
         <f>Federal_Funds_Effective_Rate!C44</f>
@@ -9182,7 +9182,7 @@
       </c>
       <c r="E45" s="23">
         <f>Inflation!C49</f>
-        <v>3.1219823862109898E-2</v>
+        <v>8.7571022727270988E-3</v>
       </c>
       <c r="F45" s="23">
         <f>Federal_Funds_Effective_Rate!C45</f>
@@ -9207,7 +9207,7 @@
       </c>
       <c r="E46" s="23">
         <f>Inflation!C50</f>
-        <v>3.1730692955065053E-2</v>
+        <v>7.2799983102519858E-3</v>
       </c>
       <c r="F46" s="23">
         <f>Federal_Funds_Effective_Rate!C46</f>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="E47" s="23">
         <f>Inflation!C51</f>
-        <v>3.1252460048807294E-2</v>
+        <v>7.2203932423269305E-3</v>
       </c>
       <c r="F47" s="23">
         <f>Federal_Funds_Effective_Rate!C47</f>
@@ -9257,7 +9257,7 @@
       </c>
       <c r="E48" s="23">
         <f>Inflation!C52</f>
-        <v>2.8174715909090799E-2</v>
+        <v>4.6287300485773879E-3</v>
       </c>
       <c r="F48" s="23">
         <f>Federal_Funds_Effective_Rate!C48</f>
@@ -9282,7 +9282,7 @@
       </c>
       <c r="E49" s="23">
         <f>Inflation!C53</f>
-        <v>2.7697788542099557E-2</v>
+        <v>8.2891819268204568E-3</v>
       </c>
       <c r="F49" s="23">
         <f>Federal_Funds_Effective_Rate!C49</f>
@@ -9307,7 +9307,7 @@
       </c>
       <c r="E50" s="23">
         <f>Inflation!C54</f>
-        <v>2.5393696659606904E-2</v>
+        <v>5.0216829831398573E-3</v>
       </c>
       <c r="F50" s="23">
         <f>Federal_Funds_Effective_Rate!C50</f>
@@ -9332,7 +9332,7 @@
       </c>
       <c r="E51" s="23">
         <f>Inflation!C55</f>
-        <v>2.3823733518389956E-2</v>
+        <v>5.6782549420586123E-3</v>
       </c>
       <c r="F51" s="23">
         <f>Federal_Funds_Effective_Rate!C51</f>
@@ -9357,7 +9357,7 @@
       </c>
       <c r="E52" s="23">
         <f>Inflation!C56</f>
-        <v>2.8549324086290451E-2</v>
+        <v>9.265723600821639E-3</v>
       </c>
       <c r="F52" s="23">
         <f>Federal_Funds_Effective_Rate!C52</f>
@@ -9382,7 +9382,7 @@
       </c>
       <c r="E53" s="23">
         <f>Inflation!C57</f>
-        <v>2.6033281495132343E-2</v>
+        <v>5.8226997985224328E-3</v>
       </c>
       <c r="F53" s="23">
         <f>Federal_Funds_Effective_Rate!C53</f>
@@ -9407,7 +9407,7 @@
       </c>
       <c r="E54" s="23">
         <f>Inflation!C58</f>
-        <v>2.8404907975460136E-2</v>
+        <v>7.3447421661647378E-3</v>
       </c>
       <c r="F54" s="23">
         <f>Federal_Funds_Effective_Rate!C54</f>
@@ -9432,7 +9432,7 @@
       </c>
       <c r="E55" s="23">
         <f>Inflation!C59</f>
-        <v>3.0955786163095765E-2</v>
+        <v>8.1727614388832828E-3</v>
       </c>
       <c r="F55" s="23">
         <f>Federal_Funds_Effective_Rate!C55</f>
@@ -9457,7 +9457,7 @@
       </c>
       <c r="E56" s="23">
         <f>Inflation!C60</f>
-        <v>2.6642041638683576E-2</v>
+        <v>5.0427350427350156E-3</v>
       </c>
       <c r="F56" s="23">
         <f>Federal_Funds_Effective_Rate!C56</f>
@@ -9482,7 +9482,7 @@
       </c>
       <c r="E57" s="23">
         <f>Inflation!C61</f>
-        <v>2.6260791763205466E-2</v>
+        <v>5.4491813144759722E-3</v>
       </c>
       <c r="F57" s="23">
         <f>Federal_Funds_Effective_Rate!C57</f>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="E58" s="23">
         <f>Inflation!C62</f>
-        <v>2.7839090059456457E-2</v>
+        <v>8.893949251789322E-3</v>
       </c>
       <c r="F58" s="23">
         <f>Federal_Funds_Effective_Rate!C58</f>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="E59" s="23">
         <f>Inflation!C63</f>
-        <v>2.8270874424720656E-2</v>
+        <v>8.5962841868353571E-3</v>
       </c>
       <c r="F59" s="23">
         <f>Federal_Funds_Effective_Rate!C59</f>
@@ -9557,7 +9557,7 @@
       </c>
       <c r="E60" s="23">
         <f>Inflation!C64</f>
-        <v>2.8999064546305096E-2</v>
+        <v>5.7544757033248439E-3</v>
       </c>
       <c r="F60" s="23">
         <f>Federal_Funds_Effective_Rate!C60</f>
@@ -9582,7 +9582,7 @@
       </c>
       <c r="E61" s="23">
         <f>Inflation!C65</f>
-        <v>3.231620039037094E-2</v>
+        <v>8.690400508582264E-3</v>
       </c>
       <c r="F61" s="23">
         <f>Federal_Funds_Effective_Rate!C61</f>
@@ -9607,7 +9607,7 @@
       </c>
       <c r="E62" s="23">
         <f>Inflation!C66</f>
-        <v>2.9445336531950719E-2</v>
+        <v>6.0882225037342877E-3</v>
       </c>
       <c r="F62" s="23">
         <f>Federal_Funds_Effective_Rate!C62</f>
@@ -9632,7 +9632,7 @@
       </c>
       <c r="E63" s="23">
         <f>Inflation!C67</f>
-        <v>2.3017902813299195E-2</v>
+        <v>2.2990233848890281E-3</v>
       </c>
       <c r="F63" s="23">
         <f>Federal_Funds_Effective_Rate!C63</f>
@@ -9657,7 +9657,7 @@
       </c>
       <c r="E64" s="23">
         <f>Inflation!C68</f>
-        <v>2.225047679593134E-2</v>
+        <v>5.0000000000000712E-3</v>
       </c>
       <c r="F64" s="23">
         <f>Federal_Funds_Effective_Rate!C64</f>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="E65" s="23">
         <f>Inflation!C69</f>
-        <v>1.890752330352247E-2</v>
+        <v>5.3917910447760578E-3</v>
       </c>
       <c r="F65" s="23">
         <f>Federal_Funds_Effective_Rate!C65</f>
@@ -9707,7 +9707,7 @@
       </c>
       <c r="E66" s="23">
         <f>Inflation!C70</f>
-        <v>1.482776117720014E-2</v>
+        <v>2.0597895674441809E-3</v>
       </c>
       <c r="F66" s="23">
         <f>Federal_Funds_Effective_Rate!C66</f>
@@ -9732,7 +9732,7 @@
       </c>
       <c r="E67" s="23">
         <f>Inflation!C71</f>
-        <v>1.5831249999999918E-2</v>
+        <v>3.2901234567900436E-3</v>
       </c>
       <c r="F67" s="23">
         <f>Federal_Funds_Effective_Rate!C67</f>
@@ -9757,7 +9757,7 @@
       </c>
       <c r="E68" s="23">
         <f>Inflation!C72</f>
-        <v>1.5963930348258572E-2</v>
+        <v>5.1312656506678845E-3</v>
       </c>
       <c r="F68" s="23">
         <f>Federal_Funds_Effective_Rate!C68</f>
@@ -9782,7 +9782,7 @@
       </c>
       <c r="E69" s="23">
         <f>Inflation!C73</f>
-        <v>1.5253576796748923E-2</v>
+        <v>4.6888294453593417E-3</v>
       </c>
       <c r="F69" s="23">
         <f>Federal_Funds_Effective_Rate!C69</f>
@@ -9807,7 +9807,7 @@
       </c>
       <c r="E70" s="23">
         <f>Inflation!C74</f>
-        <v>1.6870370370370397E-2</v>
+        <v>3.655572005629546E-3</v>
       </c>
       <c r="F70" s="23">
         <f>Federal_Funds_Effective_Rate!C70</f>
@@ -9832,7 +9832,7 @@
       </c>
       <c r="E71" s="23">
         <f>Inflation!C75</f>
-        <v>2.112801707960861E-2</v>
+        <v>7.4909095323948986E-3</v>
       </c>
       <c r="F71" s="23">
         <f>Federal_Funds_Effective_Rate!C71</f>
@@ -9857,7 +9857,7 @@
       </c>
       <c r="E72" s="23">
         <f>Inflation!C76</f>
-        <v>2.3462510788592548E-2</v>
+        <v>7.4291877300907746E-3</v>
       </c>
       <c r="F72" s="23">
         <f>Federal_Funds_Effective_Rate!C72</f>
@@ -9882,7 +9882,7 @@
       </c>
       <c r="E73" s="23">
         <f>Inflation!C77</f>
-        <v>2.6198266040345225E-2</v>
+        <v>7.3744019138756228E-3</v>
       </c>
       <c r="F73" s="23">
         <f>Federal_Funds_Effective_Rate!C73</f>
@@ -9907,7 +9907,7 @@
       </c>
       <c r="E74" s="23">
         <f>Inflation!C78</f>
-        <v>3.2579993079710746E-2</v>
+        <v>9.8971104237293266E-3</v>
       </c>
       <c r="F74" s="23">
         <f>Federal_Funds_Effective_Rate!C74</f>
@@ -9932,7 +9932,7 @@
       </c>
       <c r="E75" s="23">
         <f>Inflation!C79</f>
-        <v>3.2934258015147468E-2</v>
+        <v>7.836566725455605E-3</v>
       </c>
       <c r="F75" s="23">
         <f>Federal_Funds_Effective_Rate!C75</f>
@@ -9957,7 +9957,7 @@
       </c>
       <c r="E76" s="23">
         <f>Inflation!C80</f>
-        <v>3.4688995215311075E-2</v>
+        <v>9.1405972012390101E-3</v>
       </c>
       <c r="F76" s="23">
         <f>Federal_Funds_Effective_Rate!C76</f>
@@ -9982,7 +9982,7 @@
       </c>
       <c r="E77" s="23">
         <f>Inflation!C81</f>
-        <v>3.4435057263125464E-2</v>
+        <v>7.1271676300578273E-3</v>
       </c>
       <c r="F77" s="23">
         <f>Federal_Funds_Effective_Rate!C77</f>
@@ -10007,7 +10007,7 @@
       </c>
       <c r="E78" s="23">
         <f>Inflation!C82</f>
-        <v>3.4097589653145279E-2</v>
+        <v>9.5676479197396684E-3</v>
       </c>
       <c r="F78" s="23">
         <f>Federal_Funds_Effective_Rate!C78</f>
@@ -10032,7 +10032,7 @@
       </c>
       <c r="E79" s="23">
         <f>Inflation!C83</f>
-        <v>3.3249141063855951E-2</v>
+        <v>7.009664582148971E-3</v>
       </c>
       <c r="F79" s="23">
         <f>Federal_Funds_Effective_Rate!C79</f>
@@ -10057,7 +10057,7 @@
       </c>
       <c r="E80" s="23">
         <f>Inflation!C84</f>
-        <v>2.6780346820809306E-2</v>
+        <v>2.8227377168568248E-3</v>
       </c>
       <c r="F80" s="23">
         <f>Federal_Funds_Effective_Rate!C80</f>
@@ -10082,7 +10082,7 @@
       </c>
       <c r="E81" s="23">
         <f>Inflation!C85</f>
-        <v>1.8750753301613333E-2</v>
+        <v>-7.4873475086278886E-4</v>
       </c>
       <c r="F81" s="23">
         <f>Federal_Funds_Effective_Rate!C81</f>
@@ -10107,7 +10107,7 @@
       </c>
       <c r="E82" s="23">
         <f>Inflation!C86</f>
-        <v>1.2319499715747593E-2</v>
+        <v>3.1943661971831397E-3</v>
       </c>
       <c r="F82" s="23">
         <f>Federal_Funds_Effective_Rate!C82</f>
@@ -10132,7 +10132,7 @@
       </c>
       <c r="E83" s="23">
         <f>Inflation!C87</f>
-        <v>1.3176539662287677E-2</v>
+        <v>7.8622091684590941E-3</v>
       </c>
       <c r="F83" s="23">
         <f>Federal_Funds_Effective_Rate!C83</f>
@@ -10157,7 +10157,7 @@
       </c>
       <c r="E84" s="23">
         <f>Inflation!C88</f>
-        <v>1.5762836860267984E-2</v>
+        <v>5.3826051586084332E-3</v>
       </c>
       <c r="F84" s="23">
         <f>Federal_Funds_Effective_Rate!C84</f>
@@ -10182,7 +10182,7 @@
       </c>
       <c r="E85" s="23">
         <f>Inflation!C89</f>
-        <v>2.2535211267605635E-2</v>
+        <v>5.9135523989514516E-3</v>
       </c>
       <c r="F85" s="23">
         <f>Federal_Funds_Effective_Rate!C85</f>
@@ -10207,7 +10207,7 @@
       </c>
       <c r="E86" s="23">
         <f>Inflation!C90</f>
-        <v>2.9764077566309215E-2</v>
+        <v>1.0286501377410414E-2</v>
       </c>
       <c r="F86" s="23">
         <f>Federal_Funds_Effective_Rate!C86</f>
@@ -10232,7 +10232,7 @@
       </c>
       <c r="E87" s="23">
         <f>Inflation!C91</f>
-        <v>2.0059398106615667E-2</v>
+        <v>-1.6360631956676118E-3</v>
       </c>
       <c r="F87" s="23">
         <f>Federal_Funds_Effective_Rate!C87</f>
@@ -10257,7 +10257,7 @@
       </c>
       <c r="E88" s="23">
         <f>Inflation!C92</f>
-        <v>2.21688937167813E-2</v>
+        <v>7.4617489771503622E-3</v>
       </c>
       <c r="F88" s="23">
         <f>Federal_Funds_Effective_Rate!C88</f>
@@ -10282,7 +10282,7 @@
       </c>
       <c r="E89" s="23">
         <f>Inflation!C93</f>
-        <v>2.0016528925619888E-2</v>
+        <v>3.7954162216090239E-3</v>
       </c>
       <c r="F89" s="23">
         <f>Federal_Funds_Effective_Rate!C89</f>
@@ -10307,7 +10307,7 @@
       </c>
       <c r="E90" s="23">
         <f>Inflation!C94</f>
-        <v>1.8176662103868192E-2</v>
+        <v>8.4641852073913289E-3</v>
       </c>
       <c r="F90" s="23">
         <f>Federal_Funds_Effective_Rate!C90</f>
@@ -10332,7 +10332,7 @@
       </c>
       <c r="E91" s="23">
         <f>Inflation!C95</f>
-        <v>2.7858652842948178E-2</v>
+        <v>7.8575254418854473E-3</v>
       </c>
       <c r="F91" s="23">
         <f>Federal_Funds_Effective_Rate!C91</f>
@@ -10357,7 +10357,7 @@
       </c>
       <c r="E92" s="23">
         <f>Inflation!C96</f>
-        <v>2.6752262339169226E-2</v>
+        <v>6.3773137691518099E-3</v>
       </c>
       <c r="F92" s="23">
         <f>Federal_Funds_Effective_Rate!C92</f>
@@ -10382,7 +10382,7 @@
       </c>
       <c r="E93" s="23">
         <f>Inflation!C97</f>
-        <v>3.3851339307416808E-2</v>
+        <v>1.0735767055506057E-2</v>
       </c>
       <c r="F93" s="23">
         <f>Federal_Funds_Effective_Rate!C93</f>
@@ -10407,7 +10407,7 @@
       </c>
       <c r="E94" s="23">
         <f>Inflation!C98</f>
-        <v>3.0353508302088925E-2</v>
+        <v>5.0522466039706606E-3</v>
       </c>
       <c r="F94" s="23">
         <f>Federal_Funds_Effective_Rate!C94</f>
@@ -10432,7 +10432,7 @@
       </c>
       <c r="E95" s="23">
         <f>Inflation!C99</f>
-        <v>2.9229354775279406E-2</v>
+        <v>6.7579158587492208E-3</v>
       </c>
       <c r="F95" s="23">
         <f>Federal_Funds_Effective_Rate!C95</f>
@@ -10457,7 +10457,7 @@
       </c>
       <c r="E96" s="23">
         <f>Inflation!C100</f>
-        <v>3.8195672952520791E-2</v>
+        <v>1.5144552246897989E-2</v>
       </c>
       <c r="F96" s="23">
         <f>Federal_Funds_Effective_Rate!C96</f>
@@ -10482,7 +10482,7 @@
       </c>
       <c r="E97" s="23">
         <f>Inflation!C101</f>
-        <v>3.6745036572622708E-2</v>
+        <v>9.3234994913529937E-3</v>
       </c>
       <c r="F97" s="23">
         <f>Federal_Funds_Effective_Rate!C97</f>
@@ -10507,7 +10507,7 @@
       </c>
       <c r="E98" s="23">
         <f>Inflation!C102</f>
-        <v>3.6908617382399388E-2</v>
+        <v>5.2108268281990406E-3</v>
       </c>
       <c r="F98" s="23">
         <f>Federal_Funds_Effective_Rate!C98</f>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="E99" s="23">
         <f>Inflation!C103</f>
-        <v>3.9242617482586062E-2</v>
+        <v>9.0240490908269685E-3</v>
       </c>
       <c r="F99" s="23">
         <f>Federal_Funds_Effective_Rate!C99</f>
@@ -10557,7 +10557,7 @@
       </c>
       <c r="E100" s="23">
         <f>Inflation!C104</f>
-        <v>3.340284842319434E-2</v>
+        <v>9.4401963560842347E-3</v>
       </c>
       <c r="F100" s="23">
         <f>Federal_Funds_Effective_Rate!C100</f>
@@ -10582,7 +10582,7 @@
       </c>
       <c r="E101" s="23">
         <f>Inflation!C105</f>
-        <v>1.9653989003845157E-2</v>
+        <v>-4.1049973666983479E-3</v>
       </c>
       <c r="F101" s="23">
         <f>Federal_Funds_Effective_Rate!C101</f>
@@ -10607,7 +10607,7 @@
       </c>
       <c r="E102" s="23">
         <f>Inflation!C106</f>
-        <v>2.4314798939172867E-2</v>
+        <v>9.8056174721869831E-3</v>
       </c>
       <c r="F102" s="23">
         <f>Federal_Funds_Effective_Rate!C102</f>
@@ -10632,7 +10632,7 @@
       </c>
       <c r="E103" s="23">
         <f>Inflation!C107</f>
-        <v>2.665116487054512E-2</v>
+        <v>1.132553825672848E-2</v>
       </c>
       <c r="F103" s="23">
         <f>Federal_Funds_Effective_Rate!C103</f>
@@ -10657,7 +10657,7 @@
       </c>
       <c r="E104" s="23">
         <f>Inflation!C108</f>
-        <v>2.3488066467487294E-2</v>
+        <v>6.3301247150717591E-3</v>
       </c>
       <c r="F104" s="23">
         <f>Federal_Funds_Effective_Rate!C104</f>
@@ -10682,7 +10682,7 @@
       </c>
       <c r="E105" s="23">
         <f>Inflation!C109</f>
-        <v>4.031472868983315E-2</v>
+        <v>1.2268020909978486E-2</v>
       </c>
       <c r="F105" s="23">
         <f>Federal_Funds_Effective_Rate!C105</f>
@@ -10707,7 +10707,7 @@
       </c>
       <c r="E106" s="23">
         <f>Inflation!C110</f>
-        <v>4.1371985688904996E-2</v>
+        <v>1.0831868497315792E-2</v>
       </c>
       <c r="F106" s="23">
         <f>Federal_Funds_Effective_Rate!C106</f>
@@ -10732,7 +10732,7 @@
       </c>
       <c r="E107" s="23">
         <f>Inflation!C111</f>
-        <v>4.3105826328092157E-2</v>
+        <v>1.3009352822296379E-2</v>
       </c>
       <c r="F107" s="23">
         <f>Federal_Funds_Effective_Rate!C107</f>
@@ -10757,7 +10757,7 @@
       </c>
       <c r="E108" s="23">
         <f>Inflation!C112</f>
-        <v>5.2525019356638232E-2</v>
+        <v>1.5417235011923554E-2</v>
       </c>
       <c r="F108" s="23">
         <f>Federal_Funds_Effective_Rate!C108</f>
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E109" s="23">
         <f>Inflation!C113</f>
-        <v>1.5958002755475226E-2</v>
+        <v>-2.2900379693047188E-2</v>
       </c>
       <c r="F109" s="23">
         <f>Federal_Funds_Effective_Rate!C109</f>
@@ -10807,7 +10807,7 @@
       </c>
       <c r="E110" s="23">
         <f>Inflation!C114</f>
-        <v>-1.8423649950652079E-3</v>
+        <v>-6.8786854275680676E-3</v>
       </c>
       <c r="F110" s="23">
         <f>Federal_Funds_Effective_Rate!C110</f>
@@ -10832,7 +10832,7 @@
       </c>
       <c r="E111" s="23">
         <f>Inflation!C115</f>
-        <v>-9.4229323831528811E-3</v>
+        <v>5.3159931819680905E-3</v>
       </c>
       <c r="F111" s="23">
         <f>Federal_Funds_Effective_Rate!C111</f>
@@ -10857,7 +10857,7 @@
       </c>
       <c r="E112" s="23">
         <f>Inflation!C116</f>
-        <v>-1.6069560131773117E-2</v>
+        <v>8.6039333604986685E-3</v>
       </c>
       <c r="F112" s="23">
         <f>Federal_Funds_Effective_Rate!C112</f>
@@ -10882,7 +10882,7 @@
       </c>
       <c r="E113" s="23">
         <f>Inflation!C117</f>
-        <v>1.4874981879737627E-2</v>
+        <v>7.8293335314659658E-3</v>
       </c>
       <c r="F113" s="23">
         <f>Federal_Funds_Effective_Rate!C113</f>
@@ -10907,7 +10907,7 @@
       </c>
       <c r="E114" s="23">
         <f>Inflation!C118</f>
-        <v>2.3524093832694579E-2</v>
+        <v>1.5850343270515325E-3</v>
       </c>
       <c r="F114" s="23">
         <f>Federal_Funds_Effective_Rate!C114</f>
@@ -10932,7 +10932,7 @@
       </c>
       <c r="E115" s="23">
         <f>Inflation!C119</f>
-        <v>1.7751174434561826E-2</v>
+        <v>-3.5422819656443817E-4</v>
       </c>
       <c r="F115" s="23">
         <f>Federal_Funds_Effective_Rate!C115</f>
@@ -10957,7 +10957,7 @@
       </c>
       <c r="E116" s="23">
         <f>Inflation!C120</f>
-        <v>1.2027267999108419E-2</v>
+        <v>2.9314716724114943E-3</v>
       </c>
       <c r="F116" s="23">
         <f>Federal_Funds_Effective_Rate!C116</f>
@@ -10982,7 +10982,7 @@
       </c>
       <c r="E117" s="23">
         <f>Inflation!C121</f>
-        <v>1.2297839008432065E-2</v>
+        <v>8.0987822001156989E-3</v>
       </c>
       <c r="F117" s="23">
         <f>Federal_Funds_Effective_Rate!C117</f>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="E118" s="23">
         <f>Inflation!C122</f>
-        <v>2.1483710103324297E-2</v>
+        <v>1.0673694463789088E-2</v>
       </c>
       <c r="F118" s="23">
         <f>Federal_Funds_Effective_Rate!C118</f>
@@ -11032,7 +11032,7 @@
       </c>
       <c r="E119" s="23">
         <f>Inflation!C123</f>
-        <v>3.3461115431874418E-2</v>
+        <v>1.1367116427374759E-2</v>
       </c>
       <c r="F119" s="23">
         <f>Federal_Funds_Effective_Rate!C119</f>
@@ -11057,7 +11057,7 @@
       </c>
       <c r="E120" s="23">
         <f>Inflation!C124</f>
-        <v>3.7162627217414396E-2</v>
+        <v>6.5236364931779015E-3</v>
       </c>
       <c r="F120" s="23">
         <f>Federal_Funds_Effective_Rate!C120</f>
@@ -11082,7 +11082,7 @@
       </c>
       <c r="E121" s="23">
         <f>Inflation!C125</f>
-        <v>3.3445759880563794E-2</v>
+        <v>4.4860706180071498E-3</v>
       </c>
       <c r="F121" s="23">
         <f>Federal_Funds_Effective_Rate!C121</f>
@@ -11107,7 +11107,7 @@
       </c>
       <c r="E122" s="23">
         <f>Inflation!C126</f>
-        <v>2.8291689935328053E-2</v>
+        <v>5.6331948891639016E-3</v>
       </c>
       <c r="F122" s="23">
         <f>Federal_Funds_Effective_Rate!C122</f>
@@ -11132,7 +11132,7 @@
       </c>
       <c r="E123" s="23">
         <f>Inflation!C127</f>
-        <v>1.8880695379573136E-2</v>
+        <v>2.1110167041861168E-3</v>
       </c>
       <c r="F123" s="23">
         <f>Federal_Funds_Effective_Rate!C123</f>
@@ -11157,7 +11157,7 @@
       </c>
       <c r="E124" s="23">
         <f>Inflation!C128</f>
-        <v>1.6847097547703305E-2</v>
+        <v>4.5147022831370206E-3</v>
       </c>
       <c r="F124" s="23">
         <f>Federal_Funds_Effective_Rate!C124</f>
@@ -11182,7 +11182,7 @@
       </c>
       <c r="E125" s="23">
         <f>Inflation!C129</f>
-        <v>1.9035706263460881E-2</v>
+        <v>6.6480741034018803E-3</v>
       </c>
       <c r="F125" s="23">
         <f>Federal_Funds_Effective_Rate!C125</f>
@@ -11207,7 +11207,7 @@
       </c>
       <c r="E126" s="23">
         <f>Inflation!C130</f>
-        <v>1.7400558850065317E-2</v>
+        <v>4.0195531812818779E-3</v>
       </c>
       <c r="F126" s="23">
         <f>Federal_Funds_Effective_Rate!C126</f>
@@ -11232,7 +11232,7 @@
       </c>
       <c r="E127" s="23">
         <f>Inflation!C131</f>
-        <v>1.4147232614244235E-2</v>
+        <v>-1.0934183961188774E-3</v>
       </c>
       <c r="F127" s="23">
         <f>Federal_Funds_Effective_Rate!C127</f>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="E128" s="23">
         <f>Inflation!C132</f>
-        <v>1.504953424323773E-2</v>
+        <v>5.4084337089789648E-3</v>
       </c>
       <c r="F128" s="23">
         <f>Federal_Funds_Effective_Rate!C128</f>
@@ -11282,7 +11282,7 @@
       </c>
       <c r="E129" s="23">
         <f>Inflation!C133</f>
-        <v>1.20759479446253E-2</v>
+        <v>3.6990998714101992E-3</v>
       </c>
       <c r="F129" s="23">
         <f>Federal_Funds_Effective_Rate!C129</f>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E130" s="23">
         <f>Inflation!C134</f>
-        <v>1.4300535086246615E-2</v>
+        <v>6.2264320153055707E-3</v>
       </c>
       <c r="F130" s="23">
         <f>Federal_Funds_Effective_Rate!C130</f>
@@ -11332,7 +11332,7 @@
       </c>
       <c r="E131" s="23">
         <f>Inflation!C135</f>
-        <v>2.0801999612144313E-2</v>
+        <v>5.3093739522368753E-3</v>
       </c>
       <c r="F131" s="23">
         <f>Federal_Funds_Effective_Rate!C131</f>
@@ -11357,7 +11357,7 @@
       </c>
       <c r="E132" s="23">
         <f>Inflation!C136</f>
-        <v>1.7908272610372897E-2</v>
+        <v>2.5583437468337097E-3</v>
       </c>
       <c r="F132" s="23">
         <f>Federal_Funds_Effective_Rate!C132</f>
@@ -11382,7 +11382,7 @@
       </c>
       <c r="E133" s="23">
         <f>Inflation!C137</f>
-        <v>1.1637192895547094E-2</v>
+        <v>-2.484440663977309E-3</v>
       </c>
       <c r="F133" s="23">
         <f>Federal_Funds_Effective_Rate!C133</f>
@@ -11407,7 +11407,7 @@
       </c>
       <c r="E134" s="23">
         <f>Inflation!C138</f>
-        <v>-1.1289316317307013E-3</v>
+        <v>-6.4714126507041956E-3</v>
       </c>
       <c r="F134" s="23">
         <f>Federal_Funds_Effective_Rate!C134</f>
@@ -11432,7 +11432,7 @@
       </c>
       <c r="E135" s="23">
         <f>Inflation!C139</f>
-        <v>3.7150866290652275E-4</v>
+        <v>6.8194854581377848E-3</v>
       </c>
       <c r="F135" s="23">
         <f>Federal_Funds_Effective_Rate!C135</f>
@@ -11457,7 +11457,7 @@
       </c>
       <c r="E136" s="23">
         <f>Inflation!C140</f>
-        <v>1.5875154751176157E-3</v>
+        <v>3.7770087778527255E-3</v>
       </c>
       <c r="F136" s="23">
         <f>Federal_Funds_Effective_Rate!C136</f>
@@ -11482,7 +11482,7 @@
       </c>
       <c r="E137" s="23">
         <f>Inflation!C141</f>
-        <v>4.0061125932929651E-3</v>
+        <v>-7.5676357444664537E-5</v>
       </c>
       <c r="F137" s="23">
         <f>Federal_Funds_Effective_Rate!C137</f>
@@ -11507,7 +11507,7 @@
       </c>
       <c r="E138" s="23">
         <f>Inflation!C142</f>
-        <v>9.9169339933292393E-3</v>
+        <v>-6.222749193775407E-4</v>
       </c>
       <c r="F138" s="23">
         <f>Federal_Funds_Effective_Rate!C138</f>
@@ -11532,7 +11532,7 @@
       </c>
       <c r="E139" s="23">
         <f>Inflation!C143</f>
-        <v>1.1098919648885869E-2</v>
+        <v>7.9978459247167961E-3</v>
       </c>
       <c r="F139" s="23">
         <f>Federal_Funds_Effective_Rate!C139</f>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="E140" s="23">
         <f>Inflation!C144</f>
-        <v>1.1570074204872757E-2</v>
+        <v>4.2447514503944064E-3</v>
       </c>
       <c r="F140" s="23">
         <f>Federal_Funds_Effective_Rate!C140</f>
@@ -11582,7 +11582,7 @@
       </c>
       <c r="E141" s="23">
         <f>Inflation!C145</f>
-        <v>1.8071200023545547E-2</v>
+        <v>6.350604928368633E-3</v>
       </c>
       <c r="F141" s="23">
         <f>Federal_Funds_Effective_Rate!C141</f>
@@ -11607,7 +11607,7 @@
       </c>
       <c r="E142" s="23">
         <f>Inflation!C146</f>
-        <v>2.587414646870493E-2</v>
+        <v>7.0373964936915681E-3</v>
       </c>
       <c r="F142" s="23">
         <f>Federal_Funds_Effective_Rate!C142</f>
@@ -11632,7 +11632,7 @@
       </c>
       <c r="E143" s="23">
         <f>Inflation!C147</f>
-        <v>1.8907299970783425E-2</v>
+        <v>1.152399739172183E-3</v>
       </c>
       <c r="F143" s="23">
         <f>Federal_Funds_Effective_Rate!C143</f>
@@ -11657,7 +11657,7 @@
       </c>
       <c r="E144" s="23">
         <f>Inflation!C148</f>
-        <v>1.9450805670657989E-2</v>
+        <v>4.7804358512207176E-3</v>
       </c>
       <c r="F144" s="23">
         <f>Federal_Funds_Effective_Rate!C144</f>
@@ -11682,7 +11682,7 @@
       </c>
       <c r="E145" s="23">
         <f>Inflation!C149</f>
-        <v>2.1075020133396696E-2</v>
+        <v>7.9539478243852851E-3</v>
       </c>
       <c r="F145" s="23">
         <f>Federal_Funds_Effective_Rate!C145</f>
@@ -11707,7 +11707,7 @@
       </c>
       <c r="E146" s="23">
         <f>Inflation!C150</f>
-        <v>2.2486148647263171E-2</v>
+        <v>8.429124972698385E-3</v>
       </c>
       <c r="F146" s="23">
         <f>Federal_Funds_Effective_Rate!C146</f>
@@ -11732,7 +11732,7 @@
       </c>
       <c r="E147" s="23">
         <f>Inflation!C151</f>
-        <v>2.686793380304767E-2</v>
+        <v>5.4427607672006455E-3</v>
       </c>
       <c r="F147" s="23">
         <f>Federal_Funds_Effective_Rate!C147</f>
@@ -11757,7 +11757,7 @@
       </c>
       <c r="E148" s="23">
         <f>Inflation!C152</f>
-        <v>2.6087807344050033E-2</v>
+        <v>4.0170895846880069E-3</v>
       </c>
       <c r="F148" s="23">
         <f>Federal_Funds_Effective_Rate!C148</f>
@@ -11782,7 +11782,7 @@
       </c>
       <c r="E149" s="23">
         <f>Inflation!C153</f>
-        <v>2.2136564767551967E-2</v>
+        <v>4.0725348251392833E-3</v>
       </c>
       <c r="F149" s="23">
         <f>Federal_Funds_Effective_Rate!C149</f>
@@ -11807,7 +11807,7 @@
       </c>
       <c r="E150" s="23">
         <f>Inflation!C154</f>
-        <v>1.6300206159103461E-2</v>
+        <v>2.6710352932796076E-3</v>
       </c>
       <c r="F150" s="23">
         <f>Federal_Funds_Effective_Rate!C150</f>
@@ -11832,7 +11832,7 @@
       </c>
       <c r="E151" s="23">
         <f>Inflation!C155</f>
-        <v>1.8222507669170582E-2</v>
+        <v>7.3445257433323802E-3</v>
       </c>
       <c r="F151" s="23">
         <f>Federal_Funds_Effective_Rate!C151</f>
@@ -11857,7 +11857,7 @@
       </c>
       <c r="E152" s="23">
         <f>Inflation!C156</f>
-        <v>1.7494020326915251E-2</v>
+        <v>3.2987655094868285E-3</v>
       </c>
       <c r="F152" s="23">
         <f>Federal_Funds_Effective_Rate!C152</f>
@@ -11882,7 +11882,7 @@
       </c>
       <c r="E153" s="23">
         <f>Inflation!C157</f>
-        <v>2.048585142712412E-2</v>
+        <v>7.0249014990881225E-3</v>
       </c>
       <c r="F153" s="23">
         <f>Federal_Funds_Effective_Rate!C153</f>
@@ -11907,7 +11907,7 @@
       </c>
       <c r="E154" s="23">
         <f>Inflation!C158</f>
-        <v>2.1437648488866742E-2</v>
+        <v>3.606216652190125E-3</v>
       </c>
       <c r="F154" s="23">
         <f>Federal_Funds_Effective_Rate!C154</f>
@@ -11932,7 +11932,7 @@
       </c>
       <c r="E155" s="23">
         <f>Inflation!C159</f>
-        <v>4.0940735836266793E-3</v>
+        <v>-9.7597539583800606E-3</v>
       </c>
       <c r="F155" s="23">
         <f>Federal_Funds_Effective_Rate!C155</f>
@@ -11957,7 +11957,7 @@
       </c>
       <c r="E156" s="23">
         <f>Inflation!C160</f>
-        <v>1.223402801369829E-2</v>
+        <v>1.1432272564106593E-2</v>
       </c>
       <c r="F156" s="23">
         <f>Federal_Funds_Effective_Rate!C156</f>
@@ -11982,7 +11982,7 @@
       </c>
       <c r="E157" s="23">
         <f>Inflation!C161</f>
-        <v>1.2423998014642047E-2</v>
+        <v>7.2138938824636975E-3</v>
       </c>
       <c r="F157" s="23">
         <f>Federal_Funds_Effective_Rate!C157</f>
@@ -12007,7 +12007,7 @@
       </c>
       <c r="E158" s="23">
         <f>Inflation!C162</f>
-        <v>1.9024951896699747E-2</v>
+        <v>1.0149679040338403E-2</v>
       </c>
       <c r="F158" s="23">
         <f>Federal_Funds_Effective_Rate!C158</f>
@@ -12032,7 +12032,7 @@
       </c>
       <c r="E159" s="23">
         <f>Inflation!C163</f>
-        <v>4.7828258392770898E-2</v>
+        <v>1.8229936832207205E-2</v>
       </c>
       <c r="F159" s="23">
         <f>Federal_Funds_Effective_Rate!C159</f>
@@ -12057,7 +12057,7 @@
       </c>
       <c r="E160" s="23">
         <f>Inflation!C164</f>
-        <v>5.2495544359660848E-2</v>
+        <v>1.5937441817166161E-2</v>
       </c>
       <c r="F160" s="23">
         <f>Federal_Funds_Effective_Rate!C160</f>
@@ -12082,7 +12082,7 @@
       </c>
       <c r="E161" s="23">
         <f>Inflation!C165</f>
-        <v>6.7711764435524763E-2</v>
+        <v>2.1775464575010194E-2</v>
       </c>
       <c r="F161" s="23">
         <f>Federal_Funds_Effective_Rate!C161</f>
@@ -12107,7 +12107,7 @@
       </c>
       <c r="E162" s="23">
         <f>Inflation!C166</f>
-        <v>8.0245088002669218E-2</v>
+        <v>2.2007310660004057E-2</v>
       </c>
       <c r="F162" s="23">
         <f>Federal_Funds_Effective_Rate!C162</f>
@@ -12132,7 +12132,7 @@
       </c>
       <c r="E163" s="23">
         <f>Inflation!C167</f>
-        <v>8.5849934835226238E-2</v>
+        <v>2.3513018328852366E-2</v>
       </c>
       <c r="F163" s="23">
         <f>Federal_Funds_Effective_Rate!C163</f>
@@ -12157,7 +12157,7 @@
       </c>
       <c r="E164" s="23">
         <f>Inflation!C168</f>
-        <v>8.2919766887805557E-2</v>
+        <v>1.3195932854374775E-2</v>
       </c>
       <c r="F164" s="23">
         <f>Federal_Funds_Effective_Rate!C164</f>
@@ -12182,7 +12182,7 @@
       </c>
       <c r="E165" s="23">
         <f>Inflation!C169</f>
-        <v>7.0922011256550926E-2</v>
+        <v>1.0455131611457657E-2</v>
       </c>
       <c r="F165" s="23">
         <f>Federal_Funds_Effective_Rate!C165</f>
@@ -12207,7 +12207,7 @@
       </c>
       <c r="E166" s="23">
         <f>Inflation!C170</f>
-        <v>5.7296090640421793E-2</v>
+        <v>9.0037582651688718E-3</v>
       </c>
       <c r="F166" s="23">
         <f>Federal_Funds_Effective_Rate!C166</f>
@@ -12232,7 +12232,7 @@
       </c>
       <c r="E167" s="23">
         <f>Inflation!C171</f>
-        <v>4.0441693386601758E-2</v>
+        <v>7.197158317564672E-3</v>
       </c>
       <c r="F167" s="23">
         <f>Federal_Funds_Effective_Rate!C167</f>
@@ -12257,7 +12257,7 @@
       </c>
       <c r="E168" s="23">
         <f>Inflation!C172</f>
-        <v>3.5660494224123644E-2</v>
+        <v>8.5399376396678665E-3</v>
       </c>
       <c r="F168" s="23">
         <f>Federal_Funds_Effective_Rate!C168</f>
@@ -12282,7 +12282,7 @@
       </c>
       <c r="E169" s="23">
         <f>Inflation!C173</f>
-        <v>3.2333808978301279E-2</v>
+        <v>7.209409488576444E-3</v>
       </c>
       <c r="F169" s="23">
         <f>Federal_Funds_Effective_Rate!C169</f>
@@ -12307,7 +12307,7 @@
       </c>
       <c r="E170" s="23">
         <f>Inflation!C174</f>
-        <v>3.2443647711051245E-2</v>
+        <v>9.1111147163321689E-3</v>
       </c>
       <c r="F170" s="23">
         <f>Federal_Funds_Effective_Rate!C170</f>
@@ -12332,7 +12332,7 @@
       </c>
       <c r="E171" s="23">
         <f>Inflation!C175</f>
-        <v>3.1915174127713407E-2</v>
+        <v>6.6816075729174045E-3</v>
       </c>
       <c r="F171" s="23">
         <f>Federal_Funds_Effective_Rate!C171</f>
@@ -12357,7 +12357,7 @@
       </c>
       <c r="E172" s="23">
         <f>Inflation!C176</f>
-        <v>2.6576118749366825E-2</v>
+        <v>3.3218240646987955E-3</v>
       </c>
       <c r="F172" s="23">
         <f>Federal_Funds_Effective_Rate!C172</f>
@@ -12382,7 +12382,7 @@
       </c>
       <c r="E173" s="23">
         <f>Inflation!C177</f>
-        <v>2.7232758480832037E-2</v>
+        <v>7.8536614871340706E-3</v>
       </c>
       <c r="F173" s="23">
         <f>Federal_Funds_Effective_Rate!C173</f>
@@ -12407,7 +12407,7 @@
       </c>
       <c r="E174" s="23">
         <f>Inflation!C178</f>
-        <v>2.7240894782365563E-2</v>
+        <v>9.1191074835432814E-3</v>
       </c>
       <c r="F174" s="23">
         <f>Federal_Funds_Effective_Rate!C174</f>
@@ -12432,7 +12432,7 @@
       </c>
       <c r="E175" s="23">
         <f>Inflation!C179</f>
-        <v>2.4610244633177944E-2</v>
+        <v>4.1036074810234871E-3</v>
       </c>
       <c r="F175" s="23">
         <f>Federal_Funds_Effective_Rate!C175</f>
@@ -12457,7 +12457,7 @@
       </c>
       <c r="E176" s="23">
         <f>Inflation!C180</f>
-        <v>2.9014297038402505E-2</v>
+        <v>7.634373071144041E-3</v>
       </c>
       <c r="F176" s="23">
         <f>Federal_Funds_Effective_Rate!C176</f>
@@ -19976,8 +19976,8 @@
         <v>94.6</v>
       </c>
       <c r="C6">
-        <f>(B6-B2)/B2</f>
-        <v>7.5819089534076928E-2</v>
+        <f>(B6-B5)/B5</f>
+        <v>8.8837224183347923E-3</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -19988,8 +19988,8 @@
         <v>95.966999999999999</v>
       </c>
       <c r="C7">
-        <f t="shared" ref="C7:C70" si="0">(B7-B3)/B3</f>
-        <v>6.9067697483485055E-2</v>
+        <f t="shared" ref="C7:C70" si="0">(B7-B6)/B6</f>
+        <v>1.4450317124735778E-2</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -20001,7 +20001,7 @@
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
-        <v>5.8157304344998752E-2</v>
+        <v>1.7360134212802285E-2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -20013,7 +20013,7 @@
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>4.4429276824469281E-2</v>
+        <v>3.0727315559289522E-3</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -20025,7 +20025,7 @@
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>3.5940803382663908E-2</v>
+        <v>6.841411985744648E-4</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -20037,7 +20037,7 @@
       </c>
       <c r="C11">
         <f t="shared" si="0"/>
-        <v>3.2990507153500652E-2</v>
+        <v>1.1561224489795872E-2</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -20049,7 +20049,7 @@
       </c>
       <c r="C12">
         <f t="shared" si="0"/>
-        <v>2.5268095828254778E-2</v>
+        <v>9.7545721404577561E-3</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="C13">
         <f t="shared" si="0"/>
-        <v>3.2338435460978296E-2</v>
+        <v>9.99000999000999E-3</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
-        <v>4.6255102040816343E-2</v>
+        <v>1.4174085064292848E-2</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="C15">
         <f t="shared" si="0"/>
-        <v>4.4051930235138696E-2</v>
+        <v>9.4311099841026674E-3</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -20097,7 +20097,7 @@
       </c>
       <c r="C16">
         <f t="shared" si="0"/>
-        <v>4.2957042957043071E-2</v>
+        <v>8.6956521739130991E-3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -20109,7 +20109,7 @@
       </c>
       <c r="C17">
         <f t="shared" si="0"/>
-        <v>4.1543026706231487E-2</v>
+        <v>8.6206896551723321E-3</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -20121,7 +20121,7 @@
       </c>
       <c r="C18">
         <f t="shared" si="0"/>
-        <v>3.6417543620102744E-2</v>
+        <v>9.1832858499525053E-3</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -20133,7 +20133,7 @@
       </c>
       <c r="C19">
         <f t="shared" si="0"/>
-        <v>3.6067632850241588E-2</v>
+        <v>9.0903102562414316E-3</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -20145,7 +20145,7 @@
       </c>
       <c r="C20">
         <f t="shared" si="0"/>
-        <v>3.3524904214559385E-2</v>
+        <v>6.2201001557356554E-3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -20157,7 +20157,7 @@
       </c>
       <c r="C21">
         <f t="shared" si="0"/>
-        <v>3.5137701804368496E-2</v>
+        <v>1.0194624652455924E-2</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -20169,7 +20169,7 @@
       </c>
       <c r="C22">
         <f t="shared" si="0"/>
-        <v>3.105385491262572E-2</v>
+        <v>5.2018348623852576E-3</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -20181,7 +20181,7 @@
       </c>
       <c r="C23">
         <f t="shared" si="0"/>
-        <v>1.6785877481745332E-2</v>
+        <v>-4.873730228992232E-3</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -20193,7 +20193,7 @@
       </c>
       <c r="C24">
         <f t="shared" si="0"/>
-        <v>1.668211306765521E-2</v>
+        <v>6.1174139939284581E-3</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -20205,7 +20205,7 @@
       </c>
       <c r="C25">
         <f t="shared" si="0"/>
-        <v>1.3458715596330264E-2</v>
+        <v>6.9917958067456324E-3</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -20217,7 +20217,7 @@
       </c>
       <c r="C26">
         <f t="shared" si="0"/>
-        <v>2.0380223972546518E-2</v>
+        <v>1.2066952121448021E-2</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -20229,7 +20229,7 @@
       </c>
       <c r="C27">
         <f t="shared" si="0"/>
-        <v>3.6997973090715577E-2</v>
+        <v>1.1332737030411412E-2</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -20241,7 +20241,7 @@
       </c>
       <c r="C28">
         <f t="shared" si="0"/>
-        <v>4.1631722880583345E-2</v>
+        <v>1.0613176258324735E-2</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -20253,7 +20253,7 @@
       </c>
       <c r="C29">
         <f t="shared" si="0"/>
-        <v>4.4049354105751039E-2</v>
+        <v>9.3290276282741516E-3</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -20265,7 +20265,7 @@
       </c>
       <c r="C30">
         <f t="shared" si="0"/>
-        <v>3.965116279069774E-2</v>
+        <v>7.8034907615340422E-3</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -20277,7 +20277,7 @@
       </c>
       <c r="C31">
         <f t="shared" si="0"/>
-        <v>3.9799410968717662E-2</v>
+        <v>1.147694716646726E-2</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -20289,7 +20289,7 @@
       </c>
       <c r="C32">
         <f t="shared" si="0"/>
-        <v>4.1420532612215288E-2</v>
+        <v>1.2188794474640052E-2</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="C33">
         <f t="shared" si="0"/>
-        <v>4.3066598458377035E-2</v>
+        <v>1.0924369747899136E-2</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -20313,7 +20313,7 @@
       </c>
       <c r="C34">
         <f t="shared" si="0"/>
-        <v>4.6750922715579887E-2</v>
+        <v>1.136325852036579E-2</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -20325,7 +20325,7 @@
       </c>
       <c r="C35">
         <f t="shared" si="0"/>
-        <v>5.1596111153640073E-2</v>
+        <v>1.6158859838740117E-2</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -20337,7 +20337,7 @@
       </c>
       <c r="C36">
         <f t="shared" si="0"/>
-        <v>4.7058823529411715E-2</v>
+        <v>7.8215363212087285E-3</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -20349,7 +20349,7 @@
       </c>
       <c r="C37">
         <f t="shared" si="0"/>
-        <v>4.6275976724854589E-2</v>
+        <v>1.0168539325842779E-2</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -20361,7 +20361,7 @@
       </c>
       <c r="C38">
         <f t="shared" si="0"/>
-        <v>5.2323144320152427E-2</v>
+        <v>1.7208640866946717E-2</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -20373,7 +20373,7 @@
       </c>
       <c r="C39">
         <f t="shared" si="0"/>
-        <v>4.5837276455315455E-2</v>
+        <v>9.8958862168349142E-3</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -20385,7 +20385,7 @@
       </c>
       <c r="C40">
         <f t="shared" si="0"/>
-        <v>5.5642054574638791E-2</v>
+        <v>1.7269914926527265E-2</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -20397,7 +20397,7 @@
       </c>
       <c r="C41">
         <f t="shared" si="0"/>
-        <v>6.2764664288494934E-2</v>
+        <v>1.6984330928360252E-2</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -20409,7 +20409,7 @@
       </c>
       <c r="C42">
         <f t="shared" si="0"/>
-        <v>5.259581514140893E-2</v>
+        <v>7.4756853334529442E-3</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -20421,7 +20421,7 @@
       </c>
       <c r="C43">
         <f t="shared" si="0"/>
-        <v>4.8468677494199502E-2</v>
+        <v>5.9361713179043188E-3</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -20433,7 +20433,7 @@
       </c>
       <c r="C44">
         <f t="shared" si="0"/>
-        <v>3.8522652110116913E-2</v>
+        <v>7.6198484882013104E-3</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -20445,7 +20445,7 @@
       </c>
       <c r="C45">
         <f t="shared" si="0"/>
-        <v>2.964856803247444E-2</v>
+        <v>8.2942898975110532E-3</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -20457,7 +20457,7 @@
       </c>
       <c r="C46">
         <f t="shared" si="0"/>
-        <v>2.8938835174783187E-2</v>
+        <v>6.7812361598164382E-3</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -20469,7 +20469,7 @@
       </c>
       <c r="C47">
         <f t="shared" si="0"/>
-        <v>3.0730192450965182E-2</v>
+        <v>7.6874815204771322E-3</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -20481,7 +20481,7 @@
       </c>
       <c r="C48">
         <f t="shared" si="0"/>
-        <v>3.0746705710102615E-2</v>
+        <v>7.6359914980713732E-3</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -20493,7 +20493,7 @@
       </c>
       <c r="C49">
         <f t="shared" si="0"/>
-        <v>3.1219823862109898E-2</v>
+        <v>8.7571022727270988E-3</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -20505,7 +20505,7 @@
       </c>
       <c r="C50">
         <f t="shared" si="0"/>
-        <v>3.1730692955065053E-2</v>
+        <v>7.2799983102519858E-3</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -20517,7 +20517,7 @@
       </c>
       <c r="C51">
         <f t="shared" si="0"/>
-        <v>3.1252460048807294E-2</v>
+        <v>7.2203932423269305E-3</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="C52">
         <f t="shared" si="0"/>
-        <v>2.8174715909090799E-2</v>
+        <v>4.6287300485773879E-3</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -20541,7 +20541,7 @@
       </c>
       <c r="C53">
         <f t="shared" si="0"/>
-        <v>2.7697788542099557E-2</v>
+        <v>8.2891819268204568E-3</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="C54">
         <f t="shared" si="0"/>
-        <v>2.5393696659606904E-2</v>
+        <v>5.0216829831398573E-3</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -20565,7 +20565,7 @@
       </c>
       <c r="C55">
         <f t="shared" si="0"/>
-        <v>2.3823733518389956E-2</v>
+        <v>5.6782549420586123E-3</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -20577,7 +20577,7 @@
       </c>
       <c r="C56">
         <f t="shared" si="0"/>
-        <v>2.8549324086290451E-2</v>
+        <v>9.265723600821639E-3</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -20589,7 +20589,7 @@
       </c>
       <c r="C57">
         <f t="shared" si="0"/>
-        <v>2.6033281495132343E-2</v>
+        <v>5.8226997985224328E-3</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -20601,7 +20601,7 @@
       </c>
       <c r="C58">
         <f t="shared" si="0"/>
-        <v>2.8404907975460136E-2</v>
+        <v>7.3447421661647378E-3</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -20613,7 +20613,7 @@
       </c>
       <c r="C59">
         <f t="shared" si="0"/>
-        <v>3.0955786163095765E-2</v>
+        <v>8.1727614388832828E-3</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
@@ -20625,7 +20625,7 @@
       </c>
       <c r="C60">
         <f t="shared" si="0"/>
-        <v>2.6642041638683576E-2</v>
+        <v>5.0427350427350156E-3</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
@@ -20637,7 +20637,7 @@
       </c>
       <c r="C61">
         <f t="shared" si="0"/>
-        <v>2.6260791763205466E-2</v>
+        <v>5.4491813144759722E-3</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="C62">
         <f t="shared" si="0"/>
-        <v>2.7839090059456457E-2</v>
+        <v>8.893949251789322E-3</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -20661,7 +20661,7 @@
       </c>
       <c r="C63">
         <f t="shared" si="0"/>
-        <v>2.8270874424720656E-2</v>
+        <v>8.5962841868353571E-3</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -20673,7 +20673,7 @@
       </c>
       <c r="C64">
         <f t="shared" si="0"/>
-        <v>2.8999064546305096E-2</v>
+        <v>5.7544757033248439E-3</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
@@ -20685,7 +20685,7 @@
       </c>
       <c r="C65">
         <f t="shared" si="0"/>
-        <v>3.231620039037094E-2</v>
+        <v>8.690400508582264E-3</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
@@ -20697,7 +20697,7 @@
       </c>
       <c r="C66">
         <f t="shared" si="0"/>
-        <v>2.9445336531950719E-2</v>
+        <v>6.0882225037342877E-3</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
@@ -20709,7 +20709,7 @@
       </c>
       <c r="C67">
         <f t="shared" si="0"/>
-        <v>2.3017902813299195E-2</v>
+        <v>2.2990233848890281E-3</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
@@ -20721,7 +20721,7 @@
       </c>
       <c r="C68">
         <f t="shared" si="0"/>
-        <v>2.225047679593134E-2</v>
+        <v>5.0000000000000712E-3</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -20733,7 +20733,7 @@
       </c>
       <c r="C69">
         <f t="shared" si="0"/>
-        <v>1.890752330352247E-2</v>
+        <v>5.3917910447760578E-3</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -20745,7 +20745,7 @@
       </c>
       <c r="C70">
         <f t="shared" si="0"/>
-        <v>1.482776117720014E-2</v>
+        <v>2.0597895674441809E-3</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -20756,8 +20756,8 @@
         <v>162.53299999999999</v>
       </c>
       <c r="C71">
-        <f t="shared" ref="C71:C134" si="1">(B71-B67)/B67</f>
-        <v>1.5831249999999918E-2</v>
+        <f t="shared" ref="C71:C134" si="1">(B71-B70)/B70</f>
+        <v>3.2901234567900436E-3</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -20769,7 +20769,7 @@
       </c>
       <c r="C72">
         <f t="shared" si="1"/>
-        <v>1.5963930348258572E-2</v>
+        <v>5.1312656506678845E-3</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -20781,7 +20781,7 @@
       </c>
       <c r="C73">
         <f t="shared" si="1"/>
-        <v>1.5253576796748923E-2</v>
+        <v>4.6888294453593417E-3</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -20793,7 +20793,7 @@
       </c>
       <c r="C74">
         <f t="shared" si="1"/>
-        <v>1.6870370370370397E-2</v>
+        <v>3.655572005629546E-3</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -20805,7 +20805,7 @@
       </c>
       <c r="C75">
         <f t="shared" si="1"/>
-        <v>2.112801707960861E-2</v>
+        <v>7.4909095323948986E-3</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -20817,7 +20817,7 @@
       </c>
       <c r="C76">
         <f t="shared" si="1"/>
-        <v>2.3462510788592548E-2</v>
+        <v>7.4291877300907746E-3</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
@@ -20829,7 +20829,7 @@
       </c>
       <c r="C77">
         <f t="shared" si="1"/>
-        <v>2.6198266040345225E-2</v>
+        <v>7.3744019138756228E-3</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
@@ -20841,7 +20841,7 @@
       </c>
       <c r="C78">
         <f t="shared" si="1"/>
-        <v>3.2579993079710746E-2</v>
+        <v>9.8971104237293266E-3</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
@@ -20853,7 +20853,7 @@
       </c>
       <c r="C79">
         <f t="shared" si="1"/>
-        <v>3.2934258015147468E-2</v>
+        <v>7.836566725455605E-3</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
@@ -20865,7 +20865,7 @@
       </c>
       <c r="C80">
         <f t="shared" si="1"/>
-        <v>3.4688995215311075E-2</v>
+        <v>9.1405972012390101E-3</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -20877,7 +20877,7 @@
       </c>
       <c r="C81">
         <f t="shared" si="1"/>
-        <v>3.4435057263125464E-2</v>
+        <v>7.1271676300578273E-3</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
@@ -20889,7 +20889,7 @@
       </c>
       <c r="C82">
         <f t="shared" si="1"/>
-        <v>3.4097589653145279E-2</v>
+        <v>9.5676479197396684E-3</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
@@ -20901,7 +20901,7 @@
       </c>
       <c r="C83">
         <f t="shared" si="1"/>
-        <v>3.3249141063855951E-2</v>
+        <v>7.009664582148971E-3</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -20913,7 +20913,7 @@
       </c>
       <c r="C84">
         <f t="shared" si="1"/>
-        <v>2.6780346820809306E-2</v>
+        <v>2.8227377168568248E-3</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
@@ -20925,7 +20925,7 @@
       </c>
       <c r="C85">
         <f t="shared" si="1"/>
-        <v>1.8750753301613333E-2</v>
+        <v>-7.4873475086278886E-4</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
@@ -20937,7 +20937,7 @@
       </c>
       <c r="C86">
         <f t="shared" si="1"/>
-        <v>1.2319499715747593E-2</v>
+        <v>3.1943661971831397E-3</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -20949,7 +20949,7 @@
       </c>
       <c r="C87">
         <f t="shared" si="1"/>
-        <v>1.3176539662287677E-2</v>
+        <v>7.8622091684590941E-3</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -20961,7 +20961,7 @@
       </c>
       <c r="C88">
         <f t="shared" si="1"/>
-        <v>1.5762836860267984E-2</v>
+        <v>5.3826051586084332E-3</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -20973,7 +20973,7 @@
       </c>
       <c r="C89">
         <f t="shared" si="1"/>
-        <v>2.2535211267605635E-2</v>
+        <v>5.9135523989514516E-3</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="C90">
         <f t="shared" si="1"/>
-        <v>2.9764077566309215E-2</v>
+        <v>1.0286501377410414E-2</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="C91">
         <f t="shared" si="1"/>
-        <v>2.0059398106615667E-2</v>
+        <v>-1.6360631956676118E-3</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
@@ -21009,7 +21009,7 @@
       </c>
       <c r="C92">
         <f t="shared" si="1"/>
-        <v>2.21688937167813E-2</v>
+        <v>7.4617489771503622E-3</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
@@ -21021,7 +21021,7 @@
       </c>
       <c r="C93">
         <f t="shared" si="1"/>
-        <v>2.0016528925619888E-2</v>
+        <v>3.7954162216090239E-3</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -21033,7 +21033,7 @@
       </c>
       <c r="C94">
         <f t="shared" si="1"/>
-        <v>1.8176662103868192E-2</v>
+        <v>8.4641852073913289E-3</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
@@ -21045,7 +21045,7 @@
       </c>
       <c r="C95">
         <f t="shared" si="1"/>
-        <v>2.7858652842948178E-2</v>
+        <v>7.8575254418854473E-3</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -21057,7 +21057,7 @@
       </c>
       <c r="C96">
         <f t="shared" si="1"/>
-        <v>2.6752262339169226E-2</v>
+        <v>6.3773137691518099E-3</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -21069,7 +21069,7 @@
       </c>
       <c r="C97">
         <f t="shared" si="1"/>
-        <v>3.3851339307416808E-2</v>
+        <v>1.0735767055506057E-2</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -21081,7 +21081,7 @@
       </c>
       <c r="C98">
         <f t="shared" si="1"/>
-        <v>3.0353508302088925E-2</v>
+        <v>5.0522466039706606E-3</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
@@ -21093,7 +21093,7 @@
       </c>
       <c r="C99">
         <f t="shared" si="1"/>
-        <v>2.9229354775279406E-2</v>
+        <v>6.7579158587492208E-3</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="C100">
         <f t="shared" si="1"/>
-        <v>3.8195672952520791E-2</v>
+        <v>1.5144552246897989E-2</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -21117,7 +21117,7 @@
       </c>
       <c r="C101">
         <f t="shared" si="1"/>
-        <v>3.6745036572622708E-2</v>
+        <v>9.3234994913529937E-3</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
@@ -21129,7 +21129,7 @@
       </c>
       <c r="C102">
         <f t="shared" si="1"/>
-        <v>3.6908617382399388E-2</v>
+        <v>5.2108268281990406E-3</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
@@ -21141,7 +21141,7 @@
       </c>
       <c r="C103">
         <f t="shared" si="1"/>
-        <v>3.9242617482586062E-2</v>
+        <v>9.0240490908269685E-3</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
@@ -21153,7 +21153,7 @@
       </c>
       <c r="C104">
         <f t="shared" si="1"/>
-        <v>3.340284842319434E-2</v>
+        <v>9.4401963560842347E-3</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
@@ -21165,7 +21165,7 @@
       </c>
       <c r="C105">
         <f t="shared" si="1"/>
-        <v>1.9653989003845157E-2</v>
+        <v>-4.1049973666983479E-3</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
@@ -21177,7 +21177,7 @@
       </c>
       <c r="C106">
         <f t="shared" si="1"/>
-        <v>2.4314798939172867E-2</v>
+        <v>9.8056174721869831E-3</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
@@ -21189,7 +21189,7 @@
       </c>
       <c r="C107">
         <f t="shared" si="1"/>
-        <v>2.665116487054512E-2</v>
+        <v>1.132553825672848E-2</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -21201,7 +21201,7 @@
       </c>
       <c r="C108">
         <f t="shared" si="1"/>
-        <v>2.3488066467487294E-2</v>
+        <v>6.3301247150717591E-3</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="C109">
         <f t="shared" si="1"/>
-        <v>4.031472868983315E-2</v>
+        <v>1.2268020909978486E-2</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C110">
         <f t="shared" si="1"/>
-        <v>4.1371985688904996E-2</v>
+        <v>1.0831868497315792E-2</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
@@ -21237,7 +21237,7 @@
       </c>
       <c r="C111">
         <f t="shared" si="1"/>
-        <v>4.3105826328092157E-2</v>
+        <v>1.3009352822296379E-2</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
@@ -21249,7 +21249,7 @@
       </c>
       <c r="C112">
         <f t="shared" si="1"/>
-        <v>5.2525019356638232E-2</v>
+        <v>1.5417235011923554E-2</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
@@ -21261,7 +21261,7 @@
       </c>
       <c r="C113">
         <f t="shared" si="1"/>
-        <v>1.5958002755475226E-2</v>
+        <v>-2.2900379693047188E-2</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
@@ -21273,7 +21273,7 @@
       </c>
       <c r="C114">
         <f t="shared" si="1"/>
-        <v>-1.8423649950652079E-3</v>
+        <v>-6.8786854275680676E-3</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
@@ -21285,7 +21285,7 @@
       </c>
       <c r="C115">
         <f t="shared" si="1"/>
-        <v>-9.4229323831528811E-3</v>
+        <v>5.3159931819680905E-3</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
@@ -21297,7 +21297,7 @@
       </c>
       <c r="C116">
         <f t="shared" si="1"/>
-        <v>-1.6069560131773117E-2</v>
+        <v>8.6039333604986685E-3</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
@@ -21309,7 +21309,7 @@
       </c>
       <c r="C117">
         <f t="shared" si="1"/>
-        <v>1.4874981879737627E-2</v>
+        <v>7.8293335314659658E-3</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -21321,7 +21321,7 @@
       </c>
       <c r="C118">
         <f t="shared" si="1"/>
-        <v>2.3524093832694579E-2</v>
+        <v>1.5850343270515325E-3</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -21333,7 +21333,7 @@
       </c>
       <c r="C119">
         <f t="shared" si="1"/>
-        <v>1.7751174434561826E-2</v>
+        <v>-3.5422819656443817E-4</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
@@ -21345,7 +21345,7 @@
       </c>
       <c r="C120">
         <f t="shared" si="1"/>
-        <v>1.2027267999108419E-2</v>
+        <v>2.9314716724114943E-3</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
@@ -21357,7 +21357,7 @@
       </c>
       <c r="C121">
         <f t="shared" si="1"/>
-        <v>1.2297839008432065E-2</v>
+        <v>8.0987822001156989E-3</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
@@ -21369,7 +21369,7 @@
       </c>
       <c r="C122">
         <f t="shared" si="1"/>
-        <v>2.1483710103324297E-2</v>
+        <v>1.0673694463789088E-2</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
@@ -21381,7 +21381,7 @@
       </c>
       <c r="C123">
         <f t="shared" si="1"/>
-        <v>3.3461115431874418E-2</v>
+        <v>1.1367116427374759E-2</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
@@ -21393,7 +21393,7 @@
       </c>
       <c r="C124">
         <f t="shared" si="1"/>
-        <v>3.7162627217414396E-2</v>
+        <v>6.5236364931779015E-3</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -21405,7 +21405,7 @@
       </c>
       <c r="C125">
         <f t="shared" si="1"/>
-        <v>3.3445759880563794E-2</v>
+        <v>4.4860706180071498E-3</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -21417,7 +21417,7 @@
       </c>
       <c r="C126">
         <f t="shared" si="1"/>
-        <v>2.8291689935328053E-2</v>
+        <v>5.6331948891639016E-3</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -21429,7 +21429,7 @@
       </c>
       <c r="C127">
         <f t="shared" si="1"/>
-        <v>1.8880695379573136E-2</v>
+        <v>2.1110167041861168E-3</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="C128">
         <f t="shared" si="1"/>
-        <v>1.6847097547703305E-2</v>
+        <v>4.5147022831370206E-3</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="C129">
         <f t="shared" si="1"/>
-        <v>1.9035706263460881E-2</v>
+        <v>6.6480741034018803E-3</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
@@ -21465,7 +21465,7 @@
       </c>
       <c r="C130">
         <f t="shared" si="1"/>
-        <v>1.7400558850065317E-2</v>
+        <v>4.0195531812818779E-3</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
@@ -21477,7 +21477,7 @@
       </c>
       <c r="C131">
         <f t="shared" si="1"/>
-        <v>1.4147232614244235E-2</v>
+        <v>-1.0934183961188774E-3</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
@@ -21489,7 +21489,7 @@
       </c>
       <c r="C132">
         <f t="shared" si="1"/>
-        <v>1.504953424323773E-2</v>
+        <v>5.4084337089789648E-3</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
@@ -21501,7 +21501,7 @@
       </c>
       <c r="C133">
         <f t="shared" si="1"/>
-        <v>1.20759479446253E-2</v>
+        <v>3.6990998714101992E-3</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
@@ -21513,7 +21513,7 @@
       </c>
       <c r="C134">
         <f t="shared" si="1"/>
-        <v>1.4300535086246615E-2</v>
+        <v>6.2264320153055707E-3</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
@@ -21524,8 +21524,8 @@
         <v>236.87200000000001</v>
       </c>
       <c r="C135">
-        <f t="shared" ref="C135:C180" si="2">(B135-B131)/B131</f>
-        <v>2.0801999612144313E-2</v>
+        <f t="shared" ref="C135:C180" si="2">(B135-B134)/B134</f>
+        <v>5.3093739522368753E-3</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
@@ -21537,7 +21537,7 @@
       </c>
       <c r="C136">
         <f t="shared" si="2"/>
-        <v>1.7908272610372897E-2</v>
+        <v>2.5583437468337097E-3</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
@@ -21549,7 +21549,7 @@
       </c>
       <c r="C137">
         <f t="shared" si="2"/>
-        <v>1.1637192895547094E-2</v>
+        <v>-2.484440663977309E-3</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="C138">
         <f t="shared" si="2"/>
-        <v>-1.1289316317307013E-3</v>
+        <v>-6.4714126507041956E-3</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
@@ -21573,7 +21573,7 @@
       </c>
       <c r="C139">
         <f t="shared" si="2"/>
-        <v>3.7150866290652275E-4</v>
+        <v>6.8194854581377848E-3</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -21585,7 +21585,7 @@
       </c>
       <c r="C140">
         <f t="shared" si="2"/>
-        <v>1.5875154751176157E-3</v>
+        <v>3.7770087778527255E-3</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
@@ -21597,7 +21597,7 @@
       </c>
       <c r="C141">
         <f t="shared" si="2"/>
-        <v>4.0061125932929651E-3</v>
+        <v>-7.5676357444664537E-5</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
@@ -21609,7 +21609,7 @@
       </c>
       <c r="C142">
         <f t="shared" si="2"/>
-        <v>9.9169339933292393E-3</v>
+        <v>-6.222749193775407E-4</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
@@ -21621,7 +21621,7 @@
       </c>
       <c r="C143">
         <f t="shared" si="2"/>
-        <v>1.1098919648885869E-2</v>
+        <v>7.9978459247167961E-3</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -21633,7 +21633,7 @@
       </c>
       <c r="C144">
         <f t="shared" si="2"/>
-        <v>1.1570074204872757E-2</v>
+        <v>4.2447514503944064E-3</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -21645,7 +21645,7 @@
       </c>
       <c r="C145">
         <f t="shared" si="2"/>
-        <v>1.8071200023545547E-2</v>
+        <v>6.350604928368633E-3</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -21657,7 +21657,7 @@
       </c>
       <c r="C146">
         <f t="shared" si="2"/>
-        <v>2.587414646870493E-2</v>
+        <v>7.0373964936915681E-3</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.2">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="C147">
         <f t="shared" si="2"/>
-        <v>1.8907299970783425E-2</v>
+        <v>1.152399739172183E-3</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -21681,7 +21681,7 @@
       </c>
       <c r="C148">
         <f t="shared" si="2"/>
-        <v>1.9450805670657989E-2</v>
+        <v>4.7804358512207176E-3</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -21693,7 +21693,7 @@
       </c>
       <c r="C149">
         <f t="shared" si="2"/>
-        <v>2.1075020133396696E-2</v>
+        <v>7.9539478243852851E-3</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -21705,7 +21705,7 @@
       </c>
       <c r="C150">
         <f t="shared" si="2"/>
-        <v>2.2486148647263171E-2</v>
+        <v>8.429124972698385E-3</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
@@ -21717,7 +21717,7 @@
       </c>
       <c r="C151">
         <f t="shared" si="2"/>
-        <v>2.686793380304767E-2</v>
+        <v>5.4427607672006455E-3</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
@@ -21729,7 +21729,7 @@
       </c>
       <c r="C152">
         <f t="shared" si="2"/>
-        <v>2.6087807344050033E-2</v>
+        <v>4.0170895846880069E-3</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="C153">
         <f t="shared" si="2"/>
-        <v>2.2136564767551967E-2</v>
+        <v>4.0725348251392833E-3</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
@@ -21753,7 +21753,7 @@
       </c>
       <c r="C154">
         <f t="shared" si="2"/>
-        <v>1.6300206159103461E-2</v>
+        <v>2.6710352932796076E-3</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
@@ -21765,7 +21765,7 @@
       </c>
       <c r="C155">
         <f t="shared" si="2"/>
-        <v>1.8222507669170582E-2</v>
+        <v>7.3445257433323802E-3</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
@@ -21777,7 +21777,7 @@
       </c>
       <c r="C156">
         <f t="shared" si="2"/>
-        <v>1.7494020326915251E-2</v>
+        <v>3.2987655094868285E-3</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
@@ -21789,7 +21789,7 @@
       </c>
       <c r="C157">
         <f t="shared" si="2"/>
-        <v>2.048585142712412E-2</v>
+        <v>7.0249014990881225E-3</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
@@ -21801,7 +21801,7 @@
       </c>
       <c r="C158">
         <f t="shared" si="2"/>
-        <v>2.1437648488866742E-2</v>
+        <v>3.606216652190125E-3</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
@@ -21813,7 +21813,7 @@
       </c>
       <c r="C159">
         <f t="shared" si="2"/>
-        <v>4.0940735836266793E-3</v>
+        <v>-9.7597539583800606E-3</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
@@ -21825,7 +21825,7 @@
       </c>
       <c r="C160">
         <f t="shared" si="2"/>
-        <v>1.223402801369829E-2</v>
+        <v>1.1432272564106593E-2</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
@@ -21837,7 +21837,7 @@
       </c>
       <c r="C161">
         <f t="shared" si="2"/>
-        <v>1.2423998014642047E-2</v>
+        <v>7.2138938824636975E-3</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="C162">
         <f t="shared" si="2"/>
-        <v>1.9024951896699747E-2</v>
+        <v>1.0149679040338403E-2</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
@@ -21861,7 +21861,7 @@
       </c>
       <c r="C163">
         <f t="shared" si="2"/>
-        <v>4.7828258392770898E-2</v>
+        <v>1.8229936832207205E-2</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
@@ -21873,7 +21873,7 @@
       </c>
       <c r="C164">
         <f t="shared" si="2"/>
-        <v>5.2495544359660848E-2</v>
+        <v>1.5937441817166161E-2</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
@@ -21885,7 +21885,7 @@
       </c>
       <c r="C165">
         <f t="shared" si="2"/>
-        <v>6.7711764435524763E-2</v>
+        <v>2.1775464575010194E-2</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="C166">
         <f t="shared" si="2"/>
-        <v>8.0245088002669218E-2</v>
+        <v>2.2007310660004057E-2</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.2">
@@ -21909,7 +21909,7 @@
       </c>
       <c r="C167">
         <f t="shared" si="2"/>
-        <v>8.5849934835226238E-2</v>
+        <v>2.3513018328852366E-2</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
@@ -21921,7 +21921,7 @@
       </c>
       <c r="C168">
         <f t="shared" si="2"/>
-        <v>8.2919766887805557E-2</v>
+        <v>1.3195932854374775E-2</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.2">
@@ -21933,7 +21933,7 @@
       </c>
       <c r="C169">
         <f t="shared" si="2"/>
-        <v>7.0922011256550926E-2</v>
+        <v>1.0455131611457657E-2</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.2">
@@ -21945,7 +21945,7 @@
       </c>
       <c r="C170">
         <f t="shared" si="2"/>
-        <v>5.7296090640421793E-2</v>
+        <v>9.0037582651688718E-3</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.2">
@@ -21957,7 +21957,7 @@
       </c>
       <c r="C171">
         <f t="shared" si="2"/>
-        <v>4.0441693386601758E-2</v>
+        <v>7.197158317564672E-3</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.2">
@@ -21969,7 +21969,7 @@
       </c>
       <c r="C172">
         <f t="shared" si="2"/>
-        <v>3.5660494224123644E-2</v>
+        <v>8.5399376396678665E-3</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.2">
@@ -21981,7 +21981,7 @@
       </c>
       <c r="C173">
         <f t="shared" si="2"/>
-        <v>3.2333808978301279E-2</v>
+        <v>7.209409488576444E-3</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.2">
@@ -21993,7 +21993,7 @@
       </c>
       <c r="C174">
         <f t="shared" si="2"/>
-        <v>3.2443647711051245E-2</v>
+        <v>9.1111147163321689E-3</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.2">
@@ -22005,7 +22005,7 @@
       </c>
       <c r="C175">
         <f t="shared" si="2"/>
-        <v>3.1915174127713407E-2</v>
+        <v>6.6816075729174045E-3</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.2">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="C176">
         <f t="shared" si="2"/>
-        <v>2.6576118749366825E-2</v>
+        <v>3.3218240646987955E-3</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.2">
@@ -22029,7 +22029,7 @@
       </c>
       <c r="C177">
         <f t="shared" si="2"/>
-        <v>2.7232758480832037E-2</v>
+        <v>7.8536614871340706E-3</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.2">
@@ -22041,7 +22041,7 @@
       </c>
       <c r="C178">
         <f t="shared" si="2"/>
-        <v>2.7240894782365563E-2</v>
+        <v>9.1191074835432814E-3</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.2">
@@ -22053,7 +22053,7 @@
       </c>
       <c r="C179">
         <f t="shared" si="2"/>
-        <v>2.4610244633177944E-2</v>
+        <v>4.1036074810234871E-3</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.2">
@@ -22065,7 +22065,7 @@
       </c>
       <c r="C180">
         <f t="shared" si="2"/>
-        <v>2.9014297038402505E-2</v>
+        <v>7.634373071144041E-3</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>